<commit_message>
[GraFx Studio] v1.42 (#690)
</commit_message>
<xml_diff>
--- a/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
+++ b/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D195"/>
+  <dimension ref="A1:D196"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="52.5" customWidth="1" min="1" max="1"/>
@@ -955,32 +955,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drop shadows </t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C24" s="1" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D24" s="1" t="inlineStr">
+          <t xml:space="preserve">Image frame clipping masks </t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Rectangle, ellipse, polygon — with stroke and corner radius</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Frame Positioning: mm</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
+          <t xml:space="preserve">Drop shadows </t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -999,7 +999,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Frame Positioning: inch</t>
+          <t>Frame Positioning: mm</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1021,12 +1021,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Frame Positioning: pt</t>
+          <t>Frame Positioning: inch</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
@@ -1043,12 +1043,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Frame Positioning: pixels (px)</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>Frame Positioning: pt</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr">
@@ -1058,14 +1058,14 @@
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scaling </t>
+          <t>Frame Positioning: pixels (px)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1087,12 +1087,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Skewing </t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Scaling </t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C30" s="1" t="inlineStr">
@@ -1109,12 +1109,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rotating </t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t xml:space="preserve">Skewing </t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">
@@ -1131,17 +1131,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>**Text Editing**</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Rotating </t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D32" s="1" t="inlineStr">
@@ -1153,34 +1153,34 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit text inline </t>
+          <t>**Text Editing**</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D33" s="1" t="inlineStr">
         <is>
-          <t>in Template Designer Workspace</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit text story mode (with or without formatting) </t>
+          <t xml:space="preserve">Edit text inline </t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C34" s="1" t="inlineStr">
@@ -1190,19 +1190,19 @@
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>in Template Designer Workspace</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Variable-based text editing through forms </t>
+          <t xml:space="preserve">Edit text story mode (with or without formatting) </t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr">
@@ -1219,7 +1219,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paste text copied from clipboard </t>
+          <t xml:space="preserve">Variable-based text editing through forms </t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1241,12 +1241,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit text along path </t>
+          <t xml:space="preserve">Paste text copied from clipboard </t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C37" s="1" t="inlineStr">
@@ -1263,12 +1263,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Change the text color </t>
+          <t xml:space="preserve">Edit text along path </t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C38" s="1" t="inlineStr">
@@ -1285,7 +1285,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Character styles  </t>
+          <t xml:space="preserve">Change the text color </t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paragraph styles </t>
+          <t xml:space="preserve">Character styles  </t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1329,7 +1329,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bullets </t>
+          <t xml:space="preserve">Paragraph styles </t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1351,56 +1351,56 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Numbered lists</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Character style support in GraFx Studio only</t>
+          <t xml:space="preserve">Bullets </t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text wrapping around other objects </t>
-        </is>
-      </c>
-      <c r="B43" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C43" s="1" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D43" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>Numbered lists</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Character style support in GraFx Studio only</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for TrueType fonts </t>
+          <t xml:space="preserve">Text wrapping around other objects </t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C44" s="1" t="inlineStr">
@@ -1417,7 +1417,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for OpenType Fonts </t>
+          <t xml:space="preserve">Support for TrueType fonts </t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1439,7 +1439,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Support for Font Families management</t>
+          <t xml:space="preserve">Support for OpenType Fonts </t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D46" s="1" t="inlineStr">
@@ -1461,7 +1461,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Support for Font Styles management</t>
+          <t>Support for Font Families management</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1483,7 +1483,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tracking </t>
+          <t>Support for Font Styles management</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D48" s="1" t="inlineStr">
@@ -1505,7 +1505,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kerning </t>
+          <t xml:space="preserve">Tracking </t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1520,14 +1520,14 @@
       </c>
       <c r="D49" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio supports several OTF [GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GPOS Single Adjust</t>
+          <t xml:space="preserve">Kerning </t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1537,19 +1537,19 @@
       </c>
       <c r="C50" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D50" s="1" t="inlineStr">
         <is>
-          <t>[Supported GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
+          <t>GraFx Studio supports several OTF [GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>GPOS Pair Adjust</t>
+          <t>GPOS Single Adjust</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1571,7 +1571,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>GPOS Cursive</t>
+          <t>GPOS Pair Adjust</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1593,7 +1593,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GPOS Mark-to-base</t>
+          <t>GPOS Cursive</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -1615,7 +1615,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>GPOS Mark-to-ligature</t>
+          <t>GPOS Mark-to-base</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>GPOS Mark-to-Mark</t>
+          <t>GPOS Mark-to-ligature</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -1659,7 +1659,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non-Latin alphabets (Multibyte support) </t>
+          <t>GPOS Mark-to-Mark</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -1669,19 +1669,19 @@
       </c>
       <c r="C56" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D56" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>[Supported GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Right to left support </t>
+          <t xml:space="preserve">Non-Latin alphabets (Multibyte support) </t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -1696,19 +1696,19 @@
       </c>
       <c r="D57" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hyphenation </t>
+          <t xml:space="preserve">Right to left support </t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C58" s="1" t="inlineStr">
@@ -1725,12 +1725,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Baseline shift</t>
+          <t xml:space="preserve">Hyphenation </t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C59" s="1" t="inlineStr">
@@ -1747,10 +1747,10 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add strokes to text </t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
+          <t>Baseline shift</t>
+        </is>
+      </c>
+      <c r="B60" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1769,17 +1769,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Images**</t>
-        </is>
-      </c>
-      <c r="B61" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Add strokes to text </t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C61" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D61" s="1" t="inlineStr">
@@ -1791,17 +1791,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for common image formats </t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>**Images**</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
@@ -1813,7 +1813,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manual Image cropping </t>
+          <t xml:space="preserve">Support for common image formats </t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -1835,7 +1835,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automatic Image fitting </t>
+          <t xml:space="preserve">Manual Image cropping </t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -1857,7 +1857,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upload images from local client </t>
+          <t xml:space="preserve">Automatic Image fitting </t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -1879,7 +1879,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Basic image repository </t>
+          <t xml:space="preserve">Upload images from local client </t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -1901,10 +1901,10 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Link to external image repositories (e.g. DAM)</t>
-        </is>
-      </c>
-      <c r="B67" s="1" t="inlineStr">
+          <t xml:space="preserve">Basic image repository </t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1923,7 +1923,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Connector Framework</t>
+          <t>Link to external image repositories (e.g. DAM)</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D68" s="1" t="inlineStr">
@@ -1945,7 +1945,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for image transformations </t>
+          <t>Connector Framework</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -1955,19 +1955,19 @@
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio: Through Media Connectors</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for image Conversion Profiles </t>
+          <t xml:space="preserve">Support for image transformations </t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -1989,7 +1989,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Support for dynamic asset providers</t>
+          <t xml:space="preserve">Support for image Conversion Profiles </t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2011,7 +2011,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>AI powered Smart Crop</t>
+          <t>Support for dynamic asset providers</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2026,24 +2026,24 @@
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: Through Media Connectors</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>**Animation**</t>
+          <t>AI powered Smart Crop</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
@@ -2055,12 +2055,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Enable animated output</t>
+          <t>**Animation**</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
@@ -2077,7 +2077,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Define the length of the animation</t>
+          <t>Enable animated output</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2099,7 +2099,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Animate individual frames</t>
+          <t>Define the length of the animation</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2121,7 +2121,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Define intro animation</t>
+          <t>Animate individual frames</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2143,7 +2143,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Define emphasis animation</t>
+          <t>Define intro animation</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2165,7 +2165,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Define outro animation</t>
+          <t>Define emphasis animation</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2187,7 +2187,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Define ease type</t>
+          <t>Define outro animation</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2209,7 +2209,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Define tween type</t>
+          <t>Define ease type</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2231,10 +2231,10 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Maintain animation across layouts</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
+          <t>Define tween type</t>
+        </is>
+      </c>
+      <c r="B82" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2253,12 +2253,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>**Color**</t>
-        </is>
-      </c>
-      <c r="B83" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>Maintain animation across layouts</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C83" s="1" t="inlineStr">
@@ -2275,17 +2275,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for CMYK colors </t>
+          <t>**Color**</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for spot colors </t>
+          <t xml:space="preserve">Support for CMYK colors </t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2319,7 +2319,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for RGB </t>
+          <t xml:space="preserve">Support for spot colors </t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -2341,12 +2341,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for Lab colors </t>
+          <t xml:space="preserve">Support for RGB </t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C87" s="1" t="inlineStr">
@@ -2363,12 +2363,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for mixed ink colors (CMYK + Spot Colors) </t>
+          <t xml:space="preserve">Support for Lab colors </t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C88" s="1" t="inlineStr">
@@ -2385,7 +2385,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for gradients </t>
+          <t xml:space="preserve">Support for mixed ink colors (CMYK + Spot Colors) </t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -2407,7 +2407,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom colors </t>
+          <t xml:space="preserve">Support for gradients </t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -2429,17 +2429,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>**Barcodes**</t>
+          <t xml:space="preserve">Custom colors </t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
@@ -2451,17 +2451,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Pre-defined barcodes</t>
+          <t>**Barcodes**</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
@@ -2473,12 +2473,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Support for Code 25</t>
+          <t>Pre-defined barcodes</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C93" s="1" t="inlineStr">
@@ -2495,12 +2495,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Support for Code 39</t>
+          <t>Support for Code 25</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C94" s="1" t="inlineStr">
@@ -2517,12 +2517,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Support for Code 39 Extended</t>
+          <t>Support for Code 39</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C95" s="1" t="inlineStr">
@@ -2539,7 +2539,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Support for ITF14</t>
+          <t>Support for Code 39 Extended</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -2561,15 +2561,15 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Support for Code 128</t>
+          <t>Support for ITF14</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C97" s="2" t="inlineStr">
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C97" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2583,7 +2583,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for DataMatrix </t>
+          <t>Support for Code 128</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -2591,7 +2591,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="C98" s="1" t="inlineStr">
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2605,15 +2605,15 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Support for UPC-A</t>
-        </is>
-      </c>
-      <c r="B99" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C99" s="2" t="inlineStr">
+          <t xml:space="preserve">Support for DataMatrix </t>
+        </is>
+      </c>
+      <c r="B99" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C99" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2627,15 +2627,15 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Support for UPC-E</t>
-        </is>
-      </c>
-      <c r="B100" s="1" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C100" s="1" t="inlineStr">
+          <t>Support for UPC-A</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2649,7 +2649,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for EAN13 </t>
+          <t>Support for UPC-E</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -2671,10 +2671,10 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Support for EAN8</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="inlineStr">
+          <t xml:space="preserve">Support for EAN13 </t>
+        </is>
+      </c>
+      <c r="B102" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2693,10 +2693,10 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for QR </t>
-        </is>
-      </c>
-      <c r="B103" s="1" t="inlineStr">
+          <t>Support for EAN8</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2715,12 +2715,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for ISBN </t>
+          <t xml:space="preserve">Support for QR </t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C104" s="1" t="inlineStr">
@@ -2737,7 +2737,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for GS1-128 </t>
+          <t xml:space="preserve">Support for ISBN </t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -2759,7 +2759,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Support for GS1-Databar Expanded</t>
+          <t xml:space="preserve">Support for GS1-128 </t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -2781,7 +2781,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for PDF417 </t>
+          <t>Support for GS1-Databar Expanded</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -2803,7 +2803,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for Pharmacode 1-bar </t>
+          <t xml:space="preserve">Support for PDF417 </t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -2825,7 +2825,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Support for Postnet</t>
+          <t xml:space="preserve">Support for Pharmacode 1-bar </t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -2847,7 +2847,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Real-time preflight reports**</t>
+          <t>Support for Postnet</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
@@ -2869,7 +2869,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configurable preflight warnings and errors, including text overflow and resolution </t>
+          <t>**Real-time preflight reports**</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
@@ -2891,7 +2891,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Constraints**</t>
+          <t xml:space="preserve">Configurable preflight warnings and errors, including text overflow and resolution </t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
@@ -2913,7 +2913,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Document constraints </t>
+          <t>**Constraints**</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
@@ -2935,7 +2935,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page constraints </t>
+          <t xml:space="preserve">Document constraints </t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Layer constraints </t>
+          <t xml:space="preserve">Page constraints </t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -2979,12 +2979,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frame constraints </t>
+          <t xml:space="preserve">Layer constraints </t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>❇️</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
@@ -3001,12 +3001,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frame content constraints </t>
+          <t xml:space="preserve">Frame constraints </t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
@@ -3023,20 +3023,20 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Text constraints</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
+          <t xml:space="preserve">Frame content constraints </t>
+        </is>
+      </c>
+      <c r="B118" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C118" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D118" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -3045,20 +3045,20 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>**Variables**</t>
-        </is>
-      </c>
-      <c r="B119" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C119" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D119" s="1" t="inlineStr">
+          <t>Text constraints</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -3067,17 +3067,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables to insert content into templates </t>
+          <t>**Variables**</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
@@ -3089,7 +3089,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Type: Short text</t>
+          <t xml:space="preserve">Use variables to insert content into templates </t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -3111,7 +3111,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Type: Long text</t>
+          <t>Type: Short text</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -3133,12 +3133,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Type: Formatted Text</t>
+          <t>Type: Long text</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
@@ -3155,7 +3155,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Type: Structured Text</t>
+          <t>Type: Formatted Text</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -3177,12 +3177,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Type: Calculated Field</t>
+          <t>Type: Structured Text</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
@@ -3192,14 +3192,14 @@
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio: Support via JavaScript actions</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Type: Image</t>
+          <t>Type: Calculated Field</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -3214,14 +3214,14 @@
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: Support via JavaScript actions</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Type: Number</t>
+          <t>Type: Image</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -3243,7 +3243,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Type: Checkbox / Boolean</t>
+          <t>Type: Number</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -3265,7 +3265,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Type: Date</t>
+          <t>Type: Checkbox / Boolean</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Type: List</t>
+          <t>Type: Date</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -3309,12 +3309,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Type: Color</t>
+          <t>Type: List</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
@@ -3331,7 +3331,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Type: Coordinate</t>
+          <t>Type: Color</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -3353,7 +3353,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Type: Button Bar</t>
+          <t>Type: Coordinate</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -3375,12 +3375,12 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in text frames  </t>
+          <t>Type: Button Bar</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
@@ -3397,7 +3397,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in image frames </t>
+          <t xml:space="preserve">Use variables in text frames  </t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -3419,7 +3419,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in barcodes </t>
+          <t xml:space="preserve">Use variables in image frames </t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -3441,7 +3441,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in action editor  </t>
+          <t xml:space="preserve">Use variables in barcodes </t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -3463,7 +3463,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in color definitions </t>
+          <t xml:space="preserve">Use variables in action editor  </t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -3485,12 +3485,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables on layers </t>
+          <t xml:space="preserve">Use variables in color definitions </t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
@@ -3507,12 +3507,12 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add scripting intelligence to variables </t>
+          <t xml:space="preserve">Use variables on layers </t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
@@ -3522,14 +3522,14 @@
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio: Support via JavaScript actions</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create variables in document </t>
+          <t xml:space="preserve">Add scripting intelligence to variables </t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -3544,24 +3544,24 @@
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: Support via JavaScript actions</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>**Template Intelligence**</t>
+          <t xml:space="preserve">Create variables in document </t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
@@ -3573,17 +3573,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automate Artwork Production </t>
+          <t>**Template Intelligence**</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
@@ -3595,7 +3595,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Autogrow of Text frames </t>
+          <t xml:space="preserve">Automate Artwork Production </t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Copyfitting of text in variables </t>
+          <t xml:space="preserve">Autogrow of Text frames </t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -3639,7 +3639,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Copyfitting of non-variable text</t>
+          <t xml:space="preserve">Copyfitting of text in variables </t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -3649,41 +3649,41 @@
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Anchoring</t>
-        </is>
-      </c>
-      <c r="B147" s="2" t="inlineStr">
+          <t>Copyfitting of non-variable text</t>
+        </is>
+      </c>
+      <c r="B147" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Layouts</t>
+          <t>Anchoring</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -3705,7 +3705,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Inheritance model for layouts</t>
+          <t>Layouts</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
@@ -3715,7 +3715,7 @@
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
@@ -3727,7 +3727,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Layout intents defined per layout</t>
+          <t>Inheritance model for layouts</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -3749,7 +3749,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for multiple output dimensions </t>
+          <t>Layout intents defined per layout</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
@@ -3771,51 +3771,51 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Components (reusable design elements)</t>
-        </is>
-      </c>
-      <c r="B152" s="1" t="inlineStr">
+          <t xml:space="preserve">Support for multiple output dimensions </t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>Build once, reuse across templates. HTML output not supported when components are used.</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Action editor (allow scripting in your document) </t>
-        </is>
-      </c>
-      <c r="B153" s="2" t="inlineStr">
+          <t>Components (reusable design elements)</t>
+        </is>
+      </c>
+      <c r="B153" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio supports JavaScript based Actions</t>
+          <t>Build once, reuse across templates. HTML output not supported when components are used.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Event based scripting triggers  </t>
+          <t xml:space="preserve">Action editor (allow scripting in your document) </t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -3830,14 +3830,14 @@
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio supports JavaScript based Actions</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Centralized Action Management</t>
+          <t xml:space="preserve">Event based scripting triggers  </t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -3847,7 +3847,7 @@
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
@@ -3859,7 +3859,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Variable data-based scripting triggers </t>
+          <t>Centralized Action Management</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
@@ -3881,7 +3881,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>GraFx Genie (AI powered Actions)</t>
+          <t xml:space="preserve">Variable data-based scripting triggers </t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
@@ -3903,12 +3903,12 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>**Dynamic Layouts**</t>
-        </is>
-      </c>
-      <c r="B158" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Genie (AI powered Actions)</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
@@ -3925,17 +3925,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple reference points </t>
+          <t>**Dynamic Layouts**</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relative positioning of the frames </t>
+          <t xml:space="preserve">Multiple reference points </t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -3969,7 +3969,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frame positioning, resizing and rotation based on variables </t>
+          <t xml:space="preserve">Relative positioning of the frames </t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -3984,14 +3984,14 @@
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio through Actions</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flexible Document Sizes based on variables </t>
+          <t xml:space="preserve">Frame positioning, resizing and rotation based on variables </t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -4013,7 +4013,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Advanced Anchoring </t>
+          <t xml:space="preserve">Flexible Document Sizes based on variables </t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -4028,58 +4028,58 @@
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio through Actions</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>**External Assets**</t>
+          <t xml:space="preserve">Advanced Anchoring </t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use images and other assets from your DAM or asset repositories </t>
+          <t>**External Assets**</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Support for metadata mapping from PIM</t>
+          <t xml:space="preserve">Use images and other assets from your DAM or asset repositories </t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
@@ -4101,7 +4101,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Support for metadata mapping from DAM</t>
+          <t>Support for metadata mapping from PIM</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -4123,7 +4123,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Support for custom connectors (media &amp; data)</t>
+          <t>Support for metadata mapping from DAM</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -4145,12 +4145,12 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>**Data Sources**</t>
+          <t>Support for custom connectors (media &amp; data)</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
@@ -4167,17 +4167,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Connect Smart Templates to single-source-of-truth data sets and eliminate content errors. </t>
+          <t>**Data Sources**</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
@@ -4189,7 +4189,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import databases, merge data  </t>
+          <t xml:space="preserve">Connect Smart Templates to single-source-of-truth data sets and eliminate content errors. </t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -4211,7 +4211,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for structured files (csv, excel, xml) </t>
+          <t xml:space="preserve">Import databases, merge data  </t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -4233,61 +4233,61 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Data connector framework (CSV, Google Sheets)</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>Live connector-based data sources; multiple instances supported</t>
+          <t xml:space="preserve">Support for structured files (csv, excel, xml) </t>
+        </is>
+      </c>
+      <c r="B173" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C173" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D173" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>**Input**</t>
-        </is>
-      </c>
-      <c r="B174" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C174" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D174" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>Data connector framework (CSV, Google Sheets)</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Live connector-based data sources; multiple instances supported</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Import from Adobe® InDesign®</t>
-        </is>
-      </c>
-      <c r="B175" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C175" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>**Input**</t>
+        </is>
+      </c>
+      <c r="B175" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C175" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D175" s="1" t="inlineStr">
@@ -4299,7 +4299,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Import from Adobe® PhotoShop®</t>
+          <t>Import from Adobe® InDesign®</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -4307,9 +4307,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="C176" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="D176" s="1" t="inlineStr">
@@ -4321,17 +4321,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Import from Adobe® Illustrator®</t>
-        </is>
-      </c>
-      <c r="B177" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C177" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>Import from Adobe® PhotoShop®</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C177" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D177" s="1" t="inlineStr">
@@ -4343,17 +4343,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Import from Figma</t>
+          <t>Import from Adobe® Illustrator®</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
         <is>
-          <t>❇️</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D178" s="1" t="inlineStr">
@@ -4365,15 +4365,15 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>**Output**</t>
+          <t>Import from Figma</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C179" s="1" t="inlineStr">
+          <t>❇️</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -4387,17 +4387,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to PDF  </t>
+          <t>**Output**</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C180" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D180" s="1" t="inlineStr">
@@ -4409,7 +4409,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to PDF with crop  marks </t>
+          <t xml:space="preserve">Output to PDF  </t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -4431,10 +4431,10 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to PDF with variable data </t>
-        </is>
-      </c>
-      <c r="B182" s="2" t="inlineStr">
+          <t xml:space="preserve">Output to PDF with crop  marks </t>
+        </is>
+      </c>
+      <c r="B182" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -4453,10 +4453,10 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Output to JPG</t>
-        </is>
-      </c>
-      <c r="B183" s="1" t="inlineStr">
+          <t xml:space="preserve">Output to PDF with variable data </t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -4475,7 +4475,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Output to PNG</t>
+          <t>Output to JPG</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -4497,7 +4497,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Output to GIF</t>
+          <t>Output to PNG</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="C185" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D185" s="1" t="inlineStr">
@@ -4519,7 +4519,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Output to MP4</t>
+          <t>Output to GIF</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -4541,34 +4541,34 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to HTML </t>
+          <t>Output to MP4</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
         <is>
-          <t>❇️</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C187" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D187" s="1" t="inlineStr">
         <is>
-          <t>Not supported in templates that include components</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to IDML </t>
+          <t xml:space="preserve">Output to HTML </t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>❇️</t>
         </is>
       </c>
       <c r="C188" s="1" t="inlineStr">
@@ -4578,14 +4578,14 @@
       </c>
       <c r="D188" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Not supported in templates that include components</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>**Integration**</t>
+          <t xml:space="preserve">Output to IDML </t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="C189" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D189" s="1" t="inlineStr">
@@ -4607,17 +4607,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t xml:space="preserve">API-First </t>
+          <t>**Integration**</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C190" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D190" s="1" t="inlineStr">
@@ -4629,7 +4629,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>SDK Available</t>
+          <t xml:space="preserve">API-First </t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="C191" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D191" s="1" t="inlineStr">
@@ -4651,7 +4651,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open file format </t>
+          <t>SDK Available</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="C192" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D192" s="1" t="inlineStr">
@@ -4673,7 +4673,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Interfaces </t>
+          <t xml:space="preserve">Open file format </t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -4695,17 +4695,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Custom Interfaces </t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C194" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D194" s="1" t="inlineStr">
@@ -4722,15 +4722,37 @@
       </c>
       <c r="B195" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C195" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D195" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="B196" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve"> ❇️ Being developed</t>
         </is>
       </c>
-      <c r="C195" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D195" s="1" t="inlineStr">
+      <c r="C196" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D196" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>

</xml_diff>

<commit_message>
[Converter] InDesign - clipping mask support (#705)
</commit_message>
<xml_diff>
--- a/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
+++ b/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D196"/>
+  <dimension ref="A1:D197"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="52.5" customWidth="1" min="1" max="1"/>
@@ -977,32 +977,32 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drop shadows </t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C25" s="1" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D25" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>Custom shapes as image clipping masks</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Imported from [Adobe® InDesign®](/GraFx-Studio/convert/Adobe-InDesign/#clipping-mask-support)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Frame Positioning: mm</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="inlineStr">
+          <t xml:space="preserve">Drop shadows </t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1021,7 +1021,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Frame Positioning: inch</t>
+          <t>Frame Positioning: mm</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1043,12 +1043,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Frame Positioning: pt</t>
+          <t>Frame Positioning: inch</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr">
@@ -1065,12 +1065,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Frame Positioning: pixels (px)</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>Frame Positioning: pt</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
@@ -1080,14 +1080,14 @@
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scaling </t>
+          <t>Frame Positioning: pixels (px)</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1109,12 +1109,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Skewing </t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Scaling </t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">
@@ -1131,12 +1131,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rotating </t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t xml:space="preserve">Skewing </t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr">
@@ -1153,17 +1153,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>**Text Editing**</t>
-        </is>
-      </c>
-      <c r="B33" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Rotating </t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D33" s="1" t="inlineStr">
@@ -1175,34 +1175,34 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit text inline </t>
+          <t>**Text Editing**</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
-          <t>in Template Designer Workspace</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit text story mode (with or without formatting) </t>
+          <t xml:space="preserve">Edit text inline </t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr">
@@ -1212,19 +1212,19 @@
       </c>
       <c r="D35" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>in Template Designer Workspace</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Variable-based text editing through forms </t>
+          <t xml:space="preserve">Edit text story mode (with or without formatting) </t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C36" s="1" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paste text copied from clipboard </t>
+          <t xml:space="preserve">Variable-based text editing through forms </t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1263,12 +1263,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edit text along path </t>
+          <t xml:space="preserve">Paste text copied from clipboard </t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C38" s="1" t="inlineStr">
@@ -1285,12 +1285,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Change the text color </t>
+          <t xml:space="preserve">Edit text along path </t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C39" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Character styles  </t>
+          <t xml:space="preserve">Change the text color </t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1329,7 +1329,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paragraph styles </t>
+          <t xml:space="preserve">Character styles  </t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1351,7 +1351,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bullets </t>
+          <t xml:space="preserve">Paragraph styles </t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1373,56 +1373,56 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Numbered lists</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Character style support in GraFx Studio only</t>
+          <t xml:space="preserve">Bullets </t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text wrapping around other objects </t>
-        </is>
-      </c>
-      <c r="B44" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C44" s="1" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D44" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>Numbered lists</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Character style support in GraFx Studio only</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for TrueType fonts </t>
+          <t xml:space="preserve">Text wrapping around other objects </t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C45" s="1" t="inlineStr">
@@ -1439,7 +1439,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for OpenType Fonts </t>
+          <t xml:space="preserve">Support for TrueType fonts </t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1461,7 +1461,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Support for Font Families management</t>
+          <t xml:space="preserve">Support for OpenType Fonts </t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D47" s="1" t="inlineStr">
@@ -1483,7 +1483,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Support for Font Styles management</t>
+          <t>Support for Font Families management</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1505,7 +1505,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tracking </t>
+          <t>Support for Font Styles management</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="C49" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D49" s="1" t="inlineStr">
@@ -1527,7 +1527,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kerning </t>
+          <t xml:space="preserve">Tracking </t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1542,14 +1542,14 @@
       </c>
       <c r="D50" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio supports several OTF [GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>GPOS Single Adjust</t>
+          <t xml:space="preserve">Kerning </t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1559,19 +1559,19 @@
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>[Supported GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
+          <t>GraFx Studio supports several OTF [GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>GPOS Pair Adjust</t>
+          <t>GPOS Single Adjust</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1593,7 +1593,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GPOS Cursive</t>
+          <t>GPOS Pair Adjust</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -1615,7 +1615,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>GPOS Mark-to-base</t>
+          <t>GPOS Cursive</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>GPOS Mark-to-ligature</t>
+          <t>GPOS Mark-to-base</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -1659,7 +1659,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>GPOS Mark-to-Mark</t>
+          <t>GPOS Mark-to-ligature</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -1681,7 +1681,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non-Latin alphabets (Multibyte support) </t>
+          <t>GPOS Mark-to-Mark</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -1691,19 +1691,19 @@
       </c>
       <c r="C57" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D57" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>[Supported GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Right to left support </t>
+          <t xml:space="preserve">Non-Latin alphabets (Multibyte support) </t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -1718,19 +1718,19 @@
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hyphenation </t>
+          <t xml:space="preserve">Right to left support </t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C59" s="1" t="inlineStr">
@@ -1747,12 +1747,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Baseline shift</t>
+          <t xml:space="preserve">Hyphenation </t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C60" s="1" t="inlineStr">
@@ -1769,10 +1769,10 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add strokes to text </t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
+          <t>Baseline shift</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1791,17 +1791,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>**Images**</t>
-        </is>
-      </c>
-      <c r="B62" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Add strokes to text </t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
@@ -1813,17 +1813,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for common image formats </t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>**Images**</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
@@ -1835,7 +1835,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manual Image cropping </t>
+          <t xml:space="preserve">Support for common image formats </t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -1857,7 +1857,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automatic Image fitting </t>
+          <t xml:space="preserve">Manual Image cropping </t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -1879,7 +1879,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upload images from local client </t>
+          <t xml:space="preserve">Automatic Image fitting </t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -1901,7 +1901,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Basic image repository </t>
+          <t xml:space="preserve">Upload images from local client </t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -1923,10 +1923,10 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Link to external image repositories (e.g. DAM)</t>
-        </is>
-      </c>
-      <c r="B68" s="1" t="inlineStr">
+          <t xml:space="preserve">Basic image repository </t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1945,7 +1945,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Connector Framework</t>
+          <t>Link to external image repositories (e.g. DAM)</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for image transformations </t>
+          <t>Connector Framework</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -1977,19 +1977,19 @@
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio: Through Media Connectors</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for image Conversion Profiles </t>
+          <t xml:space="preserve">Support for image transformations </t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2011,7 +2011,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Support for dynamic asset providers</t>
+          <t xml:space="preserve">Support for image Conversion Profiles </t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2033,7 +2033,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>AI powered Smart Crop</t>
+          <t>Support for dynamic asset providers</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2048,24 +2048,24 @@
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: Through Media Connectors</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Animation**</t>
+          <t>AI powered Smart Crop</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
@@ -2077,12 +2077,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Enable animated output</t>
+          <t>**Animation**</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">
@@ -2099,7 +2099,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Define the length of the animation</t>
+          <t>Enable animated output</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2121,7 +2121,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Animate individual frames</t>
+          <t>Define the length of the animation</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2143,7 +2143,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Define intro animation</t>
+          <t>Animate individual frames</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2165,7 +2165,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Define emphasis animation</t>
+          <t>Define intro animation</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2187,7 +2187,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Define outro animation</t>
+          <t>Define emphasis animation</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2209,7 +2209,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Define ease type</t>
+          <t>Define outro animation</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2231,7 +2231,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Define tween type</t>
+          <t>Define ease type</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2253,10 +2253,10 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Maintain animation across layouts</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
+          <t>Define tween type</t>
+        </is>
+      </c>
+      <c r="B83" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2275,12 +2275,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>**Color**</t>
-        </is>
-      </c>
-      <c r="B84" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>Maintain animation across layouts</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C84" s="1" t="inlineStr">
@@ -2297,17 +2297,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for CMYK colors </t>
+          <t>**Color**</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
@@ -2319,7 +2319,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for spot colors </t>
+          <t xml:space="preserve">Support for CMYK colors </t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -2341,7 +2341,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for RGB </t>
+          <t xml:space="preserve">Support for spot colors </t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -2363,12 +2363,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for Lab colors </t>
+          <t xml:space="preserve">Support for RGB </t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C88" s="1" t="inlineStr">
@@ -2385,12 +2385,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for mixed ink colors (CMYK + Spot Colors) </t>
+          <t xml:space="preserve">Support for Lab colors </t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C89" s="1" t="inlineStr">
@@ -2407,7 +2407,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for gradients </t>
+          <t xml:space="preserve">Support for mixed ink colors (CMYK + Spot Colors) </t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -2429,7 +2429,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom colors </t>
+          <t xml:space="preserve">Support for gradients </t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -2451,17 +2451,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>**Barcodes**</t>
+          <t xml:space="preserve">Custom colors </t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
@@ -2473,17 +2473,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Pre-defined barcodes</t>
+          <t>**Barcodes**</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
@@ -2495,12 +2495,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Support for Code 25</t>
+          <t>Pre-defined barcodes</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C94" s="1" t="inlineStr">
@@ -2517,12 +2517,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Support for Code 39</t>
+          <t>Support for Code 25</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C95" s="1" t="inlineStr">
@@ -2539,12 +2539,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Support for Code 39 Extended</t>
+          <t>Support for Code 39</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C96" s="1" t="inlineStr">
@@ -2561,7 +2561,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Support for ITF14</t>
+          <t>Support for Code 39 Extended</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -2583,15 +2583,15 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Support for Code 128</t>
+          <t>Support for ITF14</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C98" s="2" t="inlineStr">
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C98" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2605,7 +2605,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for DataMatrix </t>
+          <t>Support for Code 128</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -2613,7 +2613,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="C99" s="1" t="inlineStr">
+      <c r="C99" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2627,15 +2627,15 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Support for UPC-A</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
+          <t xml:space="preserve">Support for DataMatrix </t>
+        </is>
+      </c>
+      <c r="B100" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C100" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2649,15 +2649,15 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Support for UPC-E</t>
-        </is>
-      </c>
-      <c r="B101" s="1" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C101" s="1" t="inlineStr">
+          <t>Support for UPC-A</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2671,7 +2671,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for EAN13 </t>
+          <t>Support for UPC-E</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -2693,10 +2693,10 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Support for EAN8</t>
-        </is>
-      </c>
-      <c r="B103" s="2" t="inlineStr">
+          <t xml:space="preserve">Support for EAN13 </t>
+        </is>
+      </c>
+      <c r="B103" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2715,10 +2715,10 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for QR </t>
-        </is>
-      </c>
-      <c r="B104" s="1" t="inlineStr">
+          <t>Support for EAN8</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2737,12 +2737,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for ISBN </t>
+          <t xml:space="preserve">Support for QR </t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C105" s="1" t="inlineStr">
@@ -2759,7 +2759,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for GS1-128 </t>
+          <t xml:space="preserve">Support for ISBN </t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -2781,7 +2781,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Support for GS1-Databar Expanded</t>
+          <t xml:space="preserve">Support for GS1-128 </t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -2803,7 +2803,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for PDF417 </t>
+          <t>Support for GS1-Databar Expanded</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -2825,7 +2825,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for Pharmacode 1-bar </t>
+          <t xml:space="preserve">Support for PDF417 </t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -2847,7 +2847,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Support for Postnet</t>
+          <t xml:space="preserve">Support for Pharmacode 1-bar </t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -2869,7 +2869,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>**Real-time preflight reports**</t>
+          <t>Support for Postnet</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
@@ -2891,7 +2891,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configurable preflight warnings and errors, including text overflow and resolution </t>
+          <t>**Real-time preflight reports**</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
@@ -2913,7 +2913,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>**Constraints**</t>
+          <t xml:space="preserve">Configurable preflight warnings and errors, including text overflow and resolution </t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
@@ -2935,7 +2935,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Document constraints </t>
+          <t>**Constraints**</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C114" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D114" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page constraints </t>
+          <t xml:space="preserve">Document constraints </t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -2979,7 +2979,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Layer constraints </t>
+          <t xml:space="preserve">Page constraints </t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3001,12 +3001,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frame constraints </t>
+          <t xml:space="preserve">Layer constraints </t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
@@ -3023,12 +3023,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frame content constraints </t>
+          <t xml:space="preserve">Frame constraints </t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
@@ -3045,20 +3045,20 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Text constraints</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
+          <t xml:space="preserve">Frame content constraints </t>
+        </is>
+      </c>
+      <c r="B119" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C119" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D119" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -3067,20 +3067,20 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>**Variables**</t>
-        </is>
-      </c>
-      <c r="B120" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C120" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D120" s="1" t="inlineStr">
+          <t>Text constraints</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -3089,17 +3089,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables to insert content into templates </t>
+          <t>**Variables**</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
@@ -3111,7 +3111,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Type: Short text</t>
+          <t xml:space="preserve">Use variables to insert content into templates </t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -3133,7 +3133,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Type: Long text</t>
+          <t>Type: Short text</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -3155,12 +3155,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Type: Formatted Text</t>
+          <t>Type: Long text</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
@@ -3177,7 +3177,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Type: Structured Text</t>
+          <t>Type: Formatted Text</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -3199,12 +3199,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Type: Calculated Field</t>
+          <t>Type: Structured Text</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
@@ -3214,14 +3214,14 @@
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio: Support via JavaScript actions</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Type: Image</t>
+          <t>Type: Calculated Field</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -3236,14 +3236,14 @@
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: Support via JavaScript actions</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Type: Number</t>
+          <t>Type: Image</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -3265,7 +3265,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Type: Checkbox / Boolean</t>
+          <t>Type: Number</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Type: Date</t>
+          <t>Type: Checkbox / Boolean</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Type: List</t>
+          <t>Type: Date</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -3331,12 +3331,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Type: Color</t>
+          <t>Type: List</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
@@ -3353,7 +3353,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Type: Coordinate</t>
+          <t>Type: Color</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -3375,7 +3375,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Type: Button Bar</t>
+          <t>Type: Coordinate</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -3397,12 +3397,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in text frames  </t>
+          <t>Type: Button Bar</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
@@ -3419,7 +3419,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in image frames </t>
+          <t xml:space="preserve">Use variables in text frames  </t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -3441,7 +3441,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in barcodes </t>
+          <t xml:space="preserve">Use variables in image frames </t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -3463,7 +3463,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in action editor  </t>
+          <t xml:space="preserve">Use variables in barcodes </t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -3485,7 +3485,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in color definitions </t>
+          <t xml:space="preserve">Use variables in action editor  </t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -3507,12 +3507,12 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables on layers </t>
+          <t xml:space="preserve">Use variables in color definitions </t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
@@ -3529,12 +3529,12 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add scripting intelligence to variables </t>
+          <t xml:space="preserve">Use variables on layers </t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
@@ -3544,14 +3544,14 @@
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio: Support via JavaScript actions</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create variables in document </t>
+          <t xml:space="preserve">Add scripting intelligence to variables </t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -3566,24 +3566,24 @@
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: Support via JavaScript actions</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>**Template Intelligence**</t>
+          <t xml:space="preserve">Create variables in document </t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
@@ -3595,17 +3595,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automate Artwork Production </t>
+          <t>**Template Intelligence**</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Autogrow of Text frames </t>
+          <t xml:space="preserve">Automate Artwork Production </t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -3639,7 +3639,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Copyfitting of text in variables </t>
+          <t xml:space="preserve">Autogrow of Text frames </t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -3661,7 +3661,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Copyfitting of non-variable text</t>
+          <t xml:space="preserve">Copyfitting of text in variables </t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -3671,41 +3671,41 @@
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Anchoring</t>
-        </is>
-      </c>
-      <c r="B148" s="2" t="inlineStr">
+          <t>Copyfitting of non-variable text</t>
+        </is>
+      </c>
+      <c r="B148" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Layouts</t>
+          <t>Anchoring</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
@@ -3727,7 +3727,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Inheritance model for layouts</t>
+          <t>Layouts</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -3737,7 +3737,7 @@
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
@@ -3749,7 +3749,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Layout intents defined per layout</t>
+          <t>Inheritance model for layouts</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -3771,7 +3771,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for multiple output dimensions </t>
+          <t>Layout intents defined per layout</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -3781,7 +3781,7 @@
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
@@ -3793,51 +3793,51 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Components (reusable design elements)</t>
-        </is>
-      </c>
-      <c r="B153" s="1" t="inlineStr">
+          <t xml:space="preserve">Support for multiple output dimensions </t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>Build once, reuse across templates. HTML output not supported when components are used.</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Action editor (allow scripting in your document) </t>
-        </is>
-      </c>
-      <c r="B154" s="2" t="inlineStr">
+          <t>Components (reusable design elements)</t>
+        </is>
+      </c>
+      <c r="B154" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio supports JavaScript based Actions</t>
+          <t>Build once, reuse across templates. HTML output not supported when components are used.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Event based scripting triggers  </t>
+          <t xml:space="preserve">Action editor (allow scripting in your document) </t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -3852,14 +3852,14 @@
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio supports JavaScript based Actions</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Centralized Action Management</t>
+          <t xml:space="preserve">Event based scripting triggers  </t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
@@ -3881,7 +3881,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Variable data-based scripting triggers </t>
+          <t>Centralized Action Management</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
@@ -3903,7 +3903,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>GraFx Genie (AI powered Actions)</t>
+          <t xml:space="preserve">Variable data-based scripting triggers </t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
@@ -3925,12 +3925,12 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>**Dynamic Layouts**</t>
-        </is>
-      </c>
-      <c r="B159" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Genie (AI powered Actions)</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
@@ -3947,17 +3947,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple reference points </t>
+          <t>**Dynamic Layouts**</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
@@ -3969,7 +3969,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relative positioning of the frames </t>
+          <t xml:space="preserve">Multiple reference points </t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -3991,7 +3991,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frame positioning, resizing and rotation based on variables </t>
+          <t xml:space="preserve">Relative positioning of the frames </t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -4006,14 +4006,14 @@
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio through Actions</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flexible Document Sizes based on variables </t>
+          <t xml:space="preserve">Frame positioning, resizing and rotation based on variables </t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -4035,7 +4035,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Advanced Anchoring </t>
+          <t xml:space="preserve">Flexible Document Sizes based on variables </t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -4050,58 +4050,58 @@
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio through Actions</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>**External Assets**</t>
+          <t xml:space="preserve">Advanced Anchoring </t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use images and other assets from your DAM or asset repositories </t>
+          <t>**External Assets**</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Support for metadata mapping from PIM</t>
+          <t xml:space="preserve">Use images and other assets from your DAM or asset repositories </t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
@@ -4123,7 +4123,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Support for metadata mapping from DAM</t>
+          <t>Support for metadata mapping from PIM</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -4145,7 +4145,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Support for custom connectors (media &amp; data)</t>
+          <t>Support for metadata mapping from DAM</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -4167,12 +4167,12 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>**Data Sources**</t>
+          <t>Support for custom connectors (media &amp; data)</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
@@ -4189,17 +4189,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Connect Smart Templates to single-source-of-truth data sets and eliminate content errors. </t>
+          <t>**Data Sources**</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C171" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D171" s="1" t="inlineStr">
@@ -4211,7 +4211,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import databases, merge data  </t>
+          <t xml:space="preserve">Connect Smart Templates to single-source-of-truth data sets and eliminate content errors. </t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -4233,7 +4233,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for structured files (csv, excel, xml) </t>
+          <t xml:space="preserve">Import databases, merge data  </t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -4255,61 +4255,61 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Data connector framework (CSV, Google Sheets)</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>Live connector-based data sources; multiple instances supported</t>
+          <t xml:space="preserve">Support for structured files (csv, excel, xml) </t>
+        </is>
+      </c>
+      <c r="B174" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C174" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D174" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>**Input**</t>
-        </is>
-      </c>
-      <c r="B175" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C175" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D175" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>Data connector framework (CSV, Google Sheets)</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Live connector-based data sources; multiple instances supported</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Import from Adobe® InDesign®</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C176" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>**Input**</t>
+        </is>
+      </c>
+      <c r="B176" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C176" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D176" s="1" t="inlineStr">
@@ -4321,7 +4321,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Import from Adobe® PhotoShop®</t>
+          <t>Import from Adobe® InDesign®</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
@@ -4329,9 +4329,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="C177" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="D177" s="1" t="inlineStr">
@@ -4343,17 +4343,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Import from Adobe® Illustrator®</t>
-        </is>
-      </c>
-      <c r="B178" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C178" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>Import from Adobe® PhotoShop®</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C178" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D178" s="1" t="inlineStr">
@@ -4365,17 +4365,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Import from Figma</t>
+          <t>Import from Adobe® Illustrator®</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
         <is>
-          <t>❇️</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D179" s="1" t="inlineStr">
@@ -4387,15 +4387,15 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>**Output**</t>
+          <t>Import from Figma</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C180" s="1" t="inlineStr">
+          <t>❇️</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -4409,17 +4409,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to PDF  </t>
+          <t>**Output**</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C181" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D181" s="1" t="inlineStr">
@@ -4431,7 +4431,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to PDF with crop  marks </t>
+          <t xml:space="preserve">Output to PDF  </t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -4453,10 +4453,10 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to PDF with variable data </t>
-        </is>
-      </c>
-      <c r="B183" s="2" t="inlineStr">
+          <t xml:space="preserve">Output to PDF with crop  marks </t>
+        </is>
+      </c>
+      <c r="B183" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -4475,10 +4475,10 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Output to JPG</t>
-        </is>
-      </c>
-      <c r="B184" s="1" t="inlineStr">
+          <t xml:space="preserve">Output to PDF with variable data </t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -4497,7 +4497,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Output to PNG</t>
+          <t>Output to JPG</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -4519,7 +4519,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Output to GIF</t>
+          <t>Output to PNG</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="C186" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D186" s="1" t="inlineStr">
@@ -4541,7 +4541,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Output to MP4</t>
+          <t>Output to GIF</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -4563,34 +4563,34 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to HTML </t>
+          <t>Output to MP4</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
         <is>
-          <t>❇️</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C188" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D188" s="1" t="inlineStr">
         <is>
-          <t>Not supported in templates that include components</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to IDML </t>
+          <t xml:space="preserve">Output to HTML </t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>❇️</t>
         </is>
       </c>
       <c r="C189" s="1" t="inlineStr">
@@ -4600,14 +4600,14 @@
       </c>
       <c r="D189" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Not supported in templates that include components</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>**Integration**</t>
+          <t xml:space="preserve">Output to IDML </t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -4617,7 +4617,7 @@
       </c>
       <c r="C190" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D190" s="1" t="inlineStr">
@@ -4629,17 +4629,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t xml:space="preserve">API-First </t>
+          <t>**Integration**</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C191" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D191" s="1" t="inlineStr">
@@ -4651,7 +4651,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>SDK Available</t>
+          <t xml:space="preserve">API-First </t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="C192" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D192" s="1" t="inlineStr">
@@ -4673,7 +4673,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open file format </t>
+          <t>SDK Available</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C193" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D193" s="1" t="inlineStr">
@@ -4695,7 +4695,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Interfaces </t>
+          <t xml:space="preserve">Open file format </t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -4717,17 +4717,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Custom Interfaces </t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C195" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D195" s="1" t="inlineStr">
@@ -4744,15 +4744,37 @@
       </c>
       <c r="B196" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C196" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D196" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="B197" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve"> ❇️ Being developed</t>
         </is>
       </c>
-      <c r="C196" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D196" s="1" t="inlineStr">
+      <c r="C197" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D197" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>

</xml_diff>

<commit_message>
[GraFx Studio] Version 1.43 (#709)
</commit_message>
<xml_diff>
--- a/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
+++ b/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D197"/>
+  <dimension ref="A1:D198"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="52.5" customWidth="1" min="1" max="1"/>
@@ -1351,7 +1351,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paragraph styles </t>
+          <t>Character style background color</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1373,7 +1373,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bullets </t>
+          <t xml:space="preserve">Paragraph styles </t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1395,56 +1395,56 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Numbered lists</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Character style support in GraFx Studio only</t>
+          <t xml:space="preserve">Bullets </t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text wrapping around other objects </t>
-        </is>
-      </c>
-      <c r="B45" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C45" s="1" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D45" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>Numbered lists</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Character style support in GraFx Studio only</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for TrueType fonts </t>
+          <t xml:space="preserve">Text wrapping around other objects </t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C46" s="1" t="inlineStr">
@@ -1461,7 +1461,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for OpenType Fonts </t>
+          <t xml:space="preserve">Support for TrueType fonts </t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1483,7 +1483,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Support for Font Families management</t>
+          <t xml:space="preserve">Support for OpenType Fonts </t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D48" s="1" t="inlineStr">
@@ -1505,7 +1505,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Support for Font Styles management</t>
+          <t>Support for Font Families management</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1527,7 +1527,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tracking </t>
+          <t>Support for Font Styles management</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="C50" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D50" s="1" t="inlineStr">
@@ -1549,7 +1549,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kerning </t>
+          <t xml:space="preserve">Tracking </t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1564,14 +1564,14 @@
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio supports several OTF [GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>GPOS Single Adjust</t>
+          <t xml:space="preserve">Kerning </t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1581,19 +1581,19 @@
       </c>
       <c r="C52" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D52" s="1" t="inlineStr">
         <is>
-          <t>[Supported GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
+          <t>GraFx Studio supports several OTF [GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GPOS Pair Adjust</t>
+          <t>GPOS Single Adjust</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -1615,7 +1615,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>GPOS Cursive</t>
+          <t>GPOS Pair Adjust</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>GPOS Mark-to-base</t>
+          <t>GPOS Cursive</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -1659,7 +1659,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>GPOS Mark-to-ligature</t>
+          <t>GPOS Mark-to-base</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -1681,7 +1681,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>GPOS Mark-to-Mark</t>
+          <t>GPOS Mark-to-ligature</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -1703,7 +1703,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non-Latin alphabets (Multibyte support) </t>
+          <t>GPOS Mark-to-Mark</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -1713,19 +1713,19 @@
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>[Supported GPOS tables](/GraFx-Fonts/overview/supported-font-types/#supported-tables)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Right to left support </t>
+          <t xml:space="preserve">Non-Latin alphabets (Multibyte support) </t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -1740,19 +1740,19 @@
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hyphenation </t>
+          <t xml:space="preserve">Right to left support </t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C60" s="1" t="inlineStr">
@@ -1769,12 +1769,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Baseline shift</t>
+          <t xml:space="preserve">Hyphenation </t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C61" s="1" t="inlineStr">
@@ -1791,10 +1791,10 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add strokes to text </t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
+          <t>Baseline shift</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1813,17 +1813,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>**Images**</t>
-        </is>
-      </c>
-      <c r="B63" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Add strokes to text </t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
@@ -1835,17 +1835,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for common image formats </t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>**Images**</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
@@ -1857,7 +1857,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manual Image cropping </t>
+          <t xml:space="preserve">Support for common image formats </t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -1879,7 +1879,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automatic Image fitting </t>
+          <t xml:space="preserve">Manual Image cropping </t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -1901,7 +1901,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upload images from local client </t>
+          <t xml:space="preserve">Automatic Image fitting </t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -1923,7 +1923,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Basic image repository </t>
+          <t xml:space="preserve">Upload images from local client </t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -1945,10 +1945,10 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Link to external image repositories (e.g. DAM)</t>
-        </is>
-      </c>
-      <c r="B69" s="1" t="inlineStr">
+          <t xml:space="preserve">Basic image repository </t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1967,7 +1967,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Connector Framework</t>
+          <t>Link to external image repositories (e.g. DAM)</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
@@ -1989,7 +1989,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for image transformations </t>
+          <t>Connector Framework</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -1999,19 +1999,19 @@
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio: Through Media Connectors</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for image Conversion Profiles </t>
+          <t xml:space="preserve">Support for image transformations </t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2033,7 +2033,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Support for dynamic asset providers</t>
+          <t xml:space="preserve">Support for image Conversion Profiles </t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2055,7 +2055,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>AI powered Smart Crop</t>
+          <t>Support for dynamic asset providers</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2070,24 +2070,24 @@
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: Through Media Connectors</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>**Animation**</t>
+          <t>AI powered Smart Crop</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
@@ -2099,12 +2099,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Enable animated output</t>
+          <t>**Animation**</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C76" s="1" t="inlineStr">
@@ -2121,7 +2121,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Define the length of the animation</t>
+          <t>Enable animated output</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2143,7 +2143,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Animate individual frames</t>
+          <t>Define the length of the animation</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2165,7 +2165,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Define intro animation</t>
+          <t>Animate individual frames</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2187,7 +2187,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Define emphasis animation</t>
+          <t>Define intro animation</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2209,7 +2209,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Define outro animation</t>
+          <t>Define emphasis animation</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2231,7 +2231,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Define ease type</t>
+          <t>Define outro animation</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2253,7 +2253,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Define tween type</t>
+          <t>Define ease type</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2275,10 +2275,10 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Maintain animation across layouts</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
+          <t>Define tween type</t>
+        </is>
+      </c>
+      <c r="B84" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2297,12 +2297,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>**Color**</t>
-        </is>
-      </c>
-      <c r="B85" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>Maintain animation across layouts</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C85" s="1" t="inlineStr">
@@ -2319,17 +2319,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for CMYK colors </t>
+          <t>**Color**</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
@@ -2341,7 +2341,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for spot colors </t>
+          <t xml:space="preserve">Support for CMYK colors </t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -2363,7 +2363,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for RGB </t>
+          <t xml:space="preserve">Support for spot colors </t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -2385,12 +2385,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for Lab colors </t>
+          <t xml:space="preserve">Support for RGB </t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C89" s="1" t="inlineStr">
@@ -2407,12 +2407,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for mixed ink colors (CMYK + Spot Colors) </t>
+          <t xml:space="preserve">Support for Lab colors </t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C90" s="1" t="inlineStr">
@@ -2429,7 +2429,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for gradients </t>
+          <t xml:space="preserve">Support for mixed ink colors (CMYK + Spot Colors) </t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -2451,7 +2451,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom colors </t>
+          <t xml:space="preserve">Support for gradients </t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -2473,17 +2473,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>**Barcodes**</t>
+          <t xml:space="preserve">Custom colors </t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
@@ -2495,17 +2495,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Pre-defined barcodes</t>
+          <t>**Barcodes**</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
@@ -2517,12 +2517,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Support for Code 25</t>
+          <t>Pre-defined barcodes</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C95" s="1" t="inlineStr">
@@ -2539,12 +2539,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Support for Code 39</t>
+          <t>Support for Code 25</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C96" s="1" t="inlineStr">
@@ -2561,12 +2561,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Support for Code 39 Extended</t>
+          <t>Support for Code 39</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C97" s="1" t="inlineStr">
@@ -2583,7 +2583,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Support for ITF14</t>
+          <t>Support for Code 39 Extended</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -2605,15 +2605,15 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Support for Code 128</t>
+          <t>Support for ITF14</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C99" s="2" t="inlineStr">
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C99" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2627,7 +2627,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for DataMatrix </t>
+          <t>Support for Code 128</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -2635,7 +2635,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="C100" s="1" t="inlineStr">
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2649,15 +2649,15 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Support for UPC-A</t>
-        </is>
-      </c>
-      <c r="B101" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C101" s="2" t="inlineStr">
+          <t xml:space="preserve">Support for DataMatrix </t>
+        </is>
+      </c>
+      <c r="B101" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C101" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2671,15 +2671,15 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Support for UPC-E</t>
-        </is>
-      </c>
-      <c r="B102" s="1" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C102" s="1" t="inlineStr">
+          <t>Support for UPC-A</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2693,7 +2693,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for EAN13 </t>
+          <t>Support for UPC-E</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -2715,10 +2715,10 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Support for EAN8</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr">
+          <t xml:space="preserve">Support for EAN13 </t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2737,10 +2737,10 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for QR </t>
-        </is>
-      </c>
-      <c r="B105" s="1" t="inlineStr">
+          <t>Support for EAN8</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2759,12 +2759,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for ISBN </t>
+          <t xml:space="preserve">Support for QR </t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C106" s="1" t="inlineStr">
@@ -2781,7 +2781,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for GS1-128 </t>
+          <t xml:space="preserve">Support for ISBN </t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -2803,7 +2803,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Support for GS1-Databar Expanded</t>
+          <t xml:space="preserve">Support for GS1-128 </t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -2825,7 +2825,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for PDF417 </t>
+          <t>Support for GS1-Databar Expanded</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -2847,7 +2847,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for Pharmacode 1-bar </t>
+          <t xml:space="preserve">Support for PDF417 </t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -2869,7 +2869,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Support for Postnet</t>
+          <t xml:space="preserve">Support for Pharmacode 1-bar </t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -2891,7 +2891,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Real-time preflight reports**</t>
+          <t>Support for Postnet</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
@@ -2913,7 +2913,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configurable preflight warnings and errors, including text overflow and resolution </t>
+          <t>**Real-time preflight reports**</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
@@ -2935,7 +2935,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Constraints**</t>
+          <t xml:space="preserve">Configurable preflight warnings and errors, including text overflow and resolution </t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C114" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D114" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Document constraints </t>
+          <t>**Constraints**</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
@@ -2979,7 +2979,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page constraints </t>
+          <t xml:space="preserve">Document constraints </t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3001,7 +3001,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Layer constraints </t>
+          <t xml:space="preserve">Page constraints </t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3023,12 +3023,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frame constraints </t>
+          <t xml:space="preserve">Layer constraints </t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
@@ -3045,12 +3045,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frame content constraints </t>
+          <t xml:space="preserve">Frame constraints </t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
@@ -3067,20 +3067,20 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Text constraints</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
+          <t xml:space="preserve">Frame content constraints </t>
+        </is>
+      </c>
+      <c r="B120" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C120" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D120" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -3089,20 +3089,20 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>**Variables**</t>
-        </is>
-      </c>
-      <c r="B121" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C121" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D121" s="1" t="inlineStr">
+          <t>Text constraints</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -3111,17 +3111,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables to insert content into templates </t>
+          <t>**Variables**</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
@@ -3133,7 +3133,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Type: Short text</t>
+          <t xml:space="preserve">Use variables to insert content into templates </t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -3155,7 +3155,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Type: Long text</t>
+          <t>Type: Short text</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -3177,12 +3177,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Type: Formatted Text</t>
+          <t>Type: Long text</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
@@ -3199,7 +3199,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Type: Structured Text</t>
+          <t>Type: Formatted Text</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -3221,12 +3221,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Type: Calculated Field</t>
+          <t>Type: Structured Text</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
@@ -3236,14 +3236,14 @@
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio: Support via JavaScript actions</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Type: Image</t>
+          <t>Type: Calculated Field</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -3258,14 +3258,14 @@
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: Support via JavaScript actions</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Type: Number</t>
+          <t>Type: Image</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Type: Checkbox / Boolean</t>
+          <t>Type: Number</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Type: Date</t>
+          <t>Type: Checkbox / Boolean</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -3331,7 +3331,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Type: List</t>
+          <t>Type: Date</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -3353,12 +3353,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Type: Color</t>
+          <t>Type: List</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
@@ -3375,7 +3375,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Type: Coordinate</t>
+          <t>Type: Color</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -3397,7 +3397,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Type: Button Bar</t>
+          <t>Type: Coordinate</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -3419,12 +3419,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in text frames  </t>
+          <t>Type: Button Bar</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
@@ -3441,7 +3441,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in image frames </t>
+          <t xml:space="preserve">Use variables in text frames  </t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -3463,7 +3463,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in barcodes </t>
+          <t xml:space="preserve">Use variables in image frames </t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -3485,7 +3485,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in action editor  </t>
+          <t xml:space="preserve">Use variables in barcodes </t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -3507,7 +3507,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables in color definitions </t>
+          <t xml:space="preserve">Use variables in action editor  </t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -3529,12 +3529,12 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use variables on layers </t>
+          <t xml:space="preserve">Use variables in color definitions </t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
@@ -3551,12 +3551,12 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add scripting intelligence to variables </t>
+          <t xml:space="preserve">Use variables on layers </t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
@@ -3566,14 +3566,14 @@
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio: Support via JavaScript actions</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Create variables in document </t>
+          <t xml:space="preserve">Add scripting intelligence to variables </t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -3588,24 +3588,24 @@
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: Support via JavaScript actions</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>**Template Intelligence**</t>
+          <t xml:space="preserve">Create variables in document </t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
@@ -3617,17 +3617,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automate Artwork Production </t>
+          <t>**Template Intelligence**</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
@@ -3639,7 +3639,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Autogrow of Text frames </t>
+          <t xml:space="preserve">Automate Artwork Production </t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -3661,7 +3661,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Copyfitting of text in variables </t>
+          <t xml:space="preserve">Autogrow of Text frames </t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -3683,7 +3683,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Copyfitting of non-variable text</t>
+          <t xml:space="preserve">Copyfitting of text in variables </t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -3693,41 +3693,41 @@
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Anchoring</t>
-        </is>
-      </c>
-      <c r="B149" s="2" t="inlineStr">
+          <t>Copyfitting of non-variable text</t>
+        </is>
+      </c>
+      <c r="B149" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Layouts</t>
+          <t>Anchoring</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -3749,7 +3749,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Inheritance model for layouts</t>
+          <t>Layouts</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
@@ -3771,7 +3771,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Layout intents defined per layout</t>
+          <t>Inheritance model for layouts</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -3793,7 +3793,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for multiple output dimensions </t>
+          <t>Layout intents defined per layout</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
@@ -3815,51 +3815,51 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Components (reusable design elements)</t>
-        </is>
-      </c>
-      <c r="B154" s="1" t="inlineStr">
+          <t xml:space="preserve">Support for multiple output dimensions </t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>Build once, reuse across templates. HTML output not supported when components are used.</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Action editor (allow scripting in your document) </t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
+          <t>Components (reusable design elements)</t>
+        </is>
+      </c>
+      <c r="B155" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio supports JavaScript based Actions</t>
+          <t>Build once, reuse across templates. HTML output not supported when components are used.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Event based scripting triggers  </t>
+          <t xml:space="preserve">Action editor (allow scripting in your document) </t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -3874,14 +3874,14 @@
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio supports JavaScript based Actions</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Centralized Action Management</t>
+          <t xml:space="preserve">Event based scripting triggers  </t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
@@ -3903,7 +3903,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Variable data-based scripting triggers </t>
+          <t>Centralized Action Management</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
@@ -3925,7 +3925,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>GraFx Genie (AI powered Actions)</t>
+          <t xml:space="preserve">Variable data-based scripting triggers </t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
@@ -3947,12 +3947,12 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>**Dynamic Layouts**</t>
-        </is>
-      </c>
-      <c r="B160" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Genie (AI powered Actions)</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
@@ -3969,17 +3969,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple reference points </t>
+          <t>**Dynamic Layouts**</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
@@ -3991,7 +3991,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relative positioning of the frames </t>
+          <t xml:space="preserve">Multiple reference points </t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -4013,7 +4013,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frame positioning, resizing and rotation based on variables </t>
+          <t xml:space="preserve">Relative positioning of the frames </t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -4028,14 +4028,14 @@
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>GraFx Studio through Actions</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flexible Document Sizes based on variables </t>
+          <t xml:space="preserve">Frame positioning, resizing and rotation based on variables </t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -4057,7 +4057,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Advanced Anchoring </t>
+          <t xml:space="preserve">Flexible Document Sizes based on variables </t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -4072,58 +4072,58 @@
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio through Actions</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>**External Assets**</t>
+          <t xml:space="preserve">Advanced Anchoring </t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use images and other assets from your DAM or asset repositories </t>
+          <t>**External Assets**</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Support for metadata mapping from PIM</t>
+          <t xml:space="preserve">Use images and other assets from your DAM or asset repositories </t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
@@ -4145,7 +4145,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Support for metadata mapping from DAM</t>
+          <t>Support for metadata mapping from PIM</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -4167,7 +4167,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Support for custom connectors (media &amp; data)</t>
+          <t>Support for metadata mapping from DAM</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -4189,12 +4189,12 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>**Data Sources**</t>
+          <t>Support for custom connectors (media &amp; data)</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C171" s="1" t="inlineStr">
@@ -4211,17 +4211,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Connect Smart Templates to single-source-of-truth data sets and eliminate content errors. </t>
+          <t>**Data Sources**</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C172" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D172" s="1" t="inlineStr">
@@ -4233,7 +4233,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import databases, merge data  </t>
+          <t xml:space="preserve">Connect Smart Templates to single-source-of-truth data sets and eliminate content errors. </t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -4255,7 +4255,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support for structured files (csv, excel, xml) </t>
+          <t xml:space="preserve">Import databases, merge data  </t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -4277,61 +4277,61 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Data connector framework (CSV, Google Sheets)</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>Live connector-based data sources; multiple instances supported</t>
+          <t xml:space="preserve">Support for structured files (csv, excel, xml) </t>
+        </is>
+      </c>
+      <c r="B175" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C175" s="1" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D175" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>**Input**</t>
-        </is>
-      </c>
-      <c r="B176" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C176" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D176" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+          <t>Data connector framework (CSV, Google Sheets)</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Live connector-based data sources; multiple instances supported</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Import from Adobe® InDesign®</t>
-        </is>
-      </c>
-      <c r="B177" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="C177" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>**Input**</t>
+        </is>
+      </c>
+      <c r="B177" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C177" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D177" s="1" t="inlineStr">
@@ -4343,7 +4343,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Import from Adobe® PhotoShop®</t>
+          <t>Import from Adobe® InDesign®</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -4351,9 +4351,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="C178" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="D178" s="1" t="inlineStr">
@@ -4365,17 +4365,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Import from Adobe® Illustrator®</t>
-        </is>
-      </c>
-      <c r="B179" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C179" s="2" t="inlineStr">
-        <is>
-          <t>✅</t>
+          <t>Import from Adobe® PhotoShop®</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C179" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D179" s="1" t="inlineStr">
@@ -4387,17 +4387,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Import from Figma</t>
+          <t>Import from Adobe® Illustrator®</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
         <is>
-          <t>❇️</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D180" s="1" t="inlineStr">
@@ -4409,15 +4409,15 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>**Output**</t>
+          <t>Import from Figma</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="C181" s="1" t="inlineStr">
+          <t>❇️</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
@@ -4431,17 +4431,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to PDF  </t>
+          <t>**Output**</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C182" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D182" s="1" t="inlineStr">
@@ -4453,7 +4453,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to PDF with crop  marks </t>
+          <t xml:space="preserve">Output to PDF  </t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -4475,10 +4475,10 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to PDF with variable data </t>
-        </is>
-      </c>
-      <c r="B184" s="2" t="inlineStr">
+          <t xml:space="preserve">Output to PDF with crop  marks </t>
+        </is>
+      </c>
+      <c r="B184" s="1" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -4497,10 +4497,10 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Output to JPG</t>
-        </is>
-      </c>
-      <c r="B185" s="1" t="inlineStr">
+          <t xml:space="preserve">Output to PDF with variable data </t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -4519,7 +4519,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Output to PNG</t>
+          <t>Output to JPG</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -4541,7 +4541,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Output to GIF</t>
+          <t>Output to PNG</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="C187" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D187" s="1" t="inlineStr">
@@ -4563,7 +4563,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Output to MP4</t>
+          <t>Output to GIF</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -4585,34 +4585,34 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to HTML </t>
+          <t>Output to MP4</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
         <is>
-          <t>❇️</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C189" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D189" s="1" t="inlineStr">
         <is>
-          <t>Not supported in templates that include components</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to IDML </t>
+          <t xml:space="preserve">Output to HTML </t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>❇️</t>
         </is>
       </c>
       <c r="C190" s="1" t="inlineStr">
@@ -4622,14 +4622,14 @@
       </c>
       <c r="D190" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Not supported in templates that include components</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>**Integration**</t>
+          <t xml:space="preserve">Output to IDML </t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="C191" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D191" s="1" t="inlineStr">
@@ -4651,17 +4651,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t xml:space="preserve">API-First </t>
+          <t>**Integration**</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C192" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D192" s="1" t="inlineStr">
@@ -4673,7 +4673,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>SDK Available</t>
+          <t xml:space="preserve">API-First </t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C193" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D193" s="1" t="inlineStr">
@@ -4695,7 +4695,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open file format </t>
+          <t>SDK Available</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="C194" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D194" s="1" t="inlineStr">
@@ -4717,7 +4717,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Interfaces </t>
+          <t xml:space="preserve">Open file format </t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -4739,17 +4739,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Custom Interfaces </t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C196" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D196" s="1" t="inlineStr">
@@ -4766,15 +4766,37 @@
       </c>
       <c r="B197" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C197" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D197" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="B198" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve"> ❇️ Being developed</t>
         </is>
       </c>
-      <c r="C197" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D197" s="1" t="inlineStr">
+      <c r="C198" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D198" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>

</xml_diff>

<commit_message>
convert RGB to CMYK
</commit_message>
<xml_diff>
--- a/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
+++ b/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D198"/>
+  <dimension ref="A1:D199"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="52.5" customWidth="1" min="1" max="1"/>
@@ -4519,10 +4519,10 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Output to JPG</t>
-        </is>
-      </c>
-      <c r="B186" s="1" t="inlineStr">
+          <t>RGB to CMYK color conversion in PDF output</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -4534,14 +4534,14 @@
       </c>
       <c r="D186" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: see [Color Management](/GraFx-Studio/guides/output/settings/#color-management)</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Output to PNG</t>
+          <t>Output to JPG</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -4563,7 +4563,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Output to GIF</t>
+          <t>Output to PNG</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -4573,7 +4573,7 @@
       </c>
       <c r="C188" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D188" s="1" t="inlineStr">
@@ -4585,7 +4585,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Output to MP4</t>
+          <t>Output to GIF</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -4607,34 +4607,34 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to HTML </t>
+          <t>Output to MP4</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
         <is>
-          <t>❇️</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C190" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D190" s="1" t="inlineStr">
         <is>
-          <t>Not supported in templates that include components</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to IDML </t>
+          <t xml:space="preserve">Output to HTML </t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>❇️</t>
         </is>
       </c>
       <c r="C191" s="1" t="inlineStr">
@@ -4644,14 +4644,14 @@
       </c>
       <c r="D191" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Not supported in templates that include components</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>**Integration**</t>
+          <t xml:space="preserve">Output to IDML </t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="C192" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D192" s="1" t="inlineStr">
@@ -4673,17 +4673,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t xml:space="preserve">API-First </t>
+          <t>**Integration**</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C193" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D193" s="1" t="inlineStr">
@@ -4695,7 +4695,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>SDK Available</t>
+          <t xml:space="preserve">API-First </t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="C194" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D194" s="1" t="inlineStr">
@@ -4717,7 +4717,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open file format </t>
+          <t>SDK Available</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="C195" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D195" s="1" t="inlineStr">
@@ -4739,7 +4739,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Interfaces </t>
+          <t xml:space="preserve">Open file format </t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -4761,17 +4761,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Custom Interfaces </t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C197" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D197" s="1" t="inlineStr">
@@ -4788,15 +4788,37 @@
       </c>
       <c r="B198" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C198" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D198" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="B199" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve"> ❇️ Being developed</t>
         </is>
       </c>
-      <c r="C198" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D198" s="1" t="inlineStr">
+      <c r="C199" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D199" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>

</xml_diff>

<commit_message>
[REL-59] convert RGB to CMYK (#766)
</commit_message>
<xml_diff>
--- a/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
+++ b/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D198"/>
+  <dimension ref="A1:D199"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="52.5" customWidth="1" min="1" max="1"/>
@@ -4519,10 +4519,10 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Output to JPG</t>
-        </is>
-      </c>
-      <c r="B186" s="1" t="inlineStr">
+          <t>RGB to CMYK color conversion in PDF output</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -4534,14 +4534,14 @@
       </c>
       <c r="D186" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: see [Color Management](/GraFx-Studio/guides/output/settings/#color-management)</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Output to PNG</t>
+          <t>Output to JPG</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -4563,7 +4563,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Output to GIF</t>
+          <t>Output to PNG</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -4573,7 +4573,7 @@
       </c>
       <c r="C188" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D188" s="1" t="inlineStr">
@@ -4585,7 +4585,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Output to MP4</t>
+          <t>Output to GIF</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -4607,34 +4607,34 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to HTML </t>
+          <t>Output to MP4</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
         <is>
-          <t>❇️</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C190" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D190" s="1" t="inlineStr">
         <is>
-          <t>Not supported in templates that include components</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t xml:space="preserve">Output to IDML </t>
+          <t xml:space="preserve">Output to HTML </t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>❇️</t>
         </is>
       </c>
       <c r="C191" s="1" t="inlineStr">
@@ -4644,14 +4644,14 @@
       </c>
       <c r="D191" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>Not supported in templates that include components</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>**Integration**</t>
+          <t xml:space="preserve">Output to IDML </t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="C192" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D192" s="1" t="inlineStr">
@@ -4673,17 +4673,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t xml:space="preserve">API-First </t>
+          <t>**Integration**</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="C193" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D193" s="1" t="inlineStr">
@@ -4695,7 +4695,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>SDK Available</t>
+          <t xml:space="preserve">API-First </t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="C194" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D194" s="1" t="inlineStr">
@@ -4717,7 +4717,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open file format </t>
+          <t>SDK Available</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="C195" s="1" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="D195" s="1" t="inlineStr">
@@ -4739,7 +4739,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Interfaces </t>
+          <t xml:space="preserve">Open file format </t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -4761,17 +4761,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t xml:space="preserve">Custom Interfaces </t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C197" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D197" s="1" t="inlineStr">
@@ -4788,15 +4788,37 @@
       </c>
       <c r="B198" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C198" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D198" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="B199" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve"> ❇️ Being developed</t>
         </is>
       </c>
-      <c r="C198" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D198" s="1" t="inlineStr">
+      <c r="C199" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D199" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>

</xml_diff>